<commit_message>
Add source and difficulty columns to Excel and data pipeline
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:O36"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -412,6 +412,8 @@
     <col min="11" max="11" width="80.83203125" customWidth="1"/>
     <col min="12" max="12" width="30.83203125" customWidth="1"/>
     <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,6 +456,12 @@
       <c r="M1" t="str">
         <v>translation</v>
       </c>
+      <c r="N1" t="str">
+        <v>source(出典、省略可)</v>
+      </c>
+      <c r="O1" t="str">
+        <v>difficulty(A〜D、省略可)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -495,6 +503,12 @@
       <c r="M2" t="str">
         <v>今出なければ遅れてしまう。</v>
       </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -536,6 +550,12 @@
       <c r="M3" t="str">
         <v>コピーしたらすぐにノートを返すよ。</v>
       </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -577,6 +597,12 @@
       <c r="M4" t="str">
         <v>指示どおりのやり方で宿題をやってこなければ、やり直しになります。</v>
       </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -618,6 +644,12 @@
       <c r="M5" t="str">
         <v>レポートを仕上げたら、帰ってもよろしい。</v>
       </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -659,6 +691,12 @@
       <c r="M6" t="str">
         <v>明日雨が降るかどうかわからない。</v>
       </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v>D</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -700,6 +738,12 @@
       <c r="M7" t="str">
         <v>そんなに長い旅の後では、お腹が空いているに違いない。</v>
       </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -741,6 +785,12 @@
       <c r="M8" t="str">
         <v>彼女は鍵を会社に忘れてきたに違いない、見つからないから。</v>
       </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -782,6 +832,12 @@
       <c r="M9" t="str">
         <v>もっと早く言ってくれればよかったのに。</v>
       </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -823,6 +879,12 @@
       <c r="M10" t="str">
         <v>窓を閉めていただけますか？少し寒いです。</v>
       </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -864,6 +926,12 @@
       <c r="M11" t="str">
         <v>嵐の間は古い橋を使うべきではない。</v>
       </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -905,6 +973,12 @@
       <c r="M12" t="str">
         <v>もっとお金があれば、あの車を買えるのに。</v>
       </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -946,6 +1020,12 @@
       <c r="M13" t="str">
         <v>去年もっと一生懸命勉強していたら、試験に合格していただろうに。</v>
       </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -987,6 +1067,12 @@
       <c r="M14" t="str">
         <v>ピアノの弾き方を知っていたらなあ。</v>
       </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1028,6 +1114,12 @@
       <c r="M15" t="str">
         <v>彼はまるで科学についてすべてを知っているかのように話す。</v>
       </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1069,6 +1161,12 @@
       <c r="M16" t="str">
         <v>あなたの助けがなければ、プロジェクトを時間通りに終わらせることはできなかっただろう。</v>
       </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1110,6 +1208,12 @@
       <c r="M17" t="str">
         <v>その小説は世界中の何百万もの読者に愛されている。</v>
       </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1151,6 +1255,12 @@
       <c r="M18" t="str">
         <v>新しい学校は来年末までに完成するだろう。</v>
       </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1192,6 +1302,12 @@
       <c r="M19" t="str">
         <v>彼女は誕生日に両親からプレゼントをもらった。</v>
       </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1233,6 +1349,12 @@
       <c r="M20" t="str">
         <v>ゲートは夜中12時前に閉められなければならない。</v>
       </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1274,6 +1396,12 @@
       <c r="M21" t="str">
         <v>英語は多くの国で公用語として話されている。</v>
       </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1315,6 +1443,12 @@
       <c r="M22" t="str">
         <v>彼女はさらなる勉強のために海外に行くことを決めた。</v>
       </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1356,6 +1490,12 @@
       <c r="M23" t="str">
         <v>決断する前に慎重に考えることが大切だ。</v>
       </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1397,6 +1537,12 @@
       <c r="M24" t="str">
         <v>彼はその答えを正確に答えた最初の生徒だった。</v>
       </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1438,6 +1584,12 @@
       <c r="M25" t="str">
         <v>彼女は成長して有名な音楽家になった。</v>
       </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1479,6 +1631,12 @@
       <c r="M26" t="str">
         <v>今は休む時間がない。</v>
       </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1520,6 +1678,12 @@
       <c r="M27" t="str">
         <v>彼はその問題に対する新しいアプローチを試してみることを提案した。</v>
       </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1561,6 +1725,12 @@
       <c r="M28" t="str">
         <v>またお会いできることを楽しみにしています。</v>
       </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1602,6 +1772,12 @@
       <c r="M29" t="str">
         <v>将来何が起こるかを知ることは不可能だ。</v>
       </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v>C</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1643,6 +1819,12 @@
       <c r="M30" t="str">
         <v>その先生は規則を厳しく守ることを主張した。</v>
       </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1684,6 +1866,12 @@
       <c r="M31" t="str">
         <v>彼女はもっと早くその間違いを犯したことを認めた。</v>
       </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+      <c r="O31" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1725,6 +1913,12 @@
       <c r="M32" t="str">
         <v>窓際に立っているあの男性は私のおじです。</v>
       </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+      <c r="O32" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1766,6 +1960,12 @@
       <c r="M33" t="str">
         <v>フランス語で書かれた手紙は理解するのが難しかった。</v>
       </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1807,6 +2007,12 @@
       <c r="M34" t="str">
         <v>丘の頂上から見ると、その街は夜に美しく見える。</v>
       </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v>B</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1848,6 +2054,12 @@
       <c r="M35" t="str">
         <v>彼女はベンチに座って本を読んでいた。</v>
       </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v>A</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1889,10 +2101,16 @@
       <c r="M36" t="str">
         <v>すべての証拠を考慮すると、陪審員は被告を無罪とした。</v>
       </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v>C</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>